<commit_message>
Add free application (M) column and badges to template, tree, detail, tables and excel export
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -413,14 +413,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,10 +442,15 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>무료원서접수</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>정원구분</t>
         </is>
@@ -466,12 +472,13 @@
           <t>인하공업전문대학</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
         <is>
           <t>https://addon.jinhakapply.com/RatioV1/RatioH/Ratio41260471.html</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>정원내</t>
         </is>
@@ -490,15 +497,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>유한대학교</t>
+          <t>경인여자대학교</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://addon.jinhakapply.com/RatioV1/RatioH/Ratio41280381.html</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
+        <is>
+          <t>https://addon.jinhakapply.com/RatioV1/RatioH/Ratio40180641.html</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>구분없음</t>
         </is>
@@ -512,20 +524,53 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>수시1차</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>연성대학교</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://addon.jinhakapply.com/RatioV1/RatioH/Ratio40580321.html</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>구분없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>수시2차</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>동양미래대학교</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>https://addon.jinhakapply.com/RatioV1/RatioH/Ratio41150241.html</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>구분없음</t>
         </is>

</xml_diff>

<commit_message>
Change free apply column value and badges from M to F
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -502,7 +502,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">

</xml_diff>

<commit_message>
feat: Add multi apply (M) column, badges, excel template and export support
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -413,15 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="65" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,10 +448,15 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>중복지원</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>정원구분</t>
         </is>
@@ -473,12 +479,13 @@
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://addon.jinhakapply.com/RatioV1/RatioH/Ratio41260471.html</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>정원내</t>
         </is>
@@ -507,10 +514,15 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>https://addon.jinhakapply.com/RatioV1/RatioH/Ratio40180641.html</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>구분없음</t>
         </is>
@@ -539,10 +551,15 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>https://addon.jinhakapply.com/RatioV1/RatioH/Ratio40580321.html</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>구분없음</t>
         </is>
@@ -565,12 +582,13 @@
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://addon.jinhakapply.com/RatioV1/RatioH/Ratio41150241.html</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>구분없음</t>
         </is>

</xml_diff>

<commit_message>
fix: Align Excel template, DB upload and UI columns to 무료접수 (F) and 중복지원 (M)
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -419,7 +419,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -443,7 +443,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>무료원서접수</t>
+          <t>무료접수</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>